<commit_message>
Pre Market Wed 2026-06-17
</commit_message>
<xml_diff>
--- a/pre-market/Pre Market 2026-06-17.xlsx
+++ b/pre-market/Pre Market 2026-06-17.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,7 +459,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7511,57</t>
+          <t>7511,34</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -476,7 +476,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>30068,18</t>
+          <t>29968,13</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -493,7 +493,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2939,23</t>
+          <t>2939,19</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>52002,93</t>
+          <t>51999,68</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4331,30</t>
+          <t>4331,18</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>69,98</t>
+          <t>70,00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1808,84</t>
+          <t>1805,60</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>79,74</t>
+          <t>78,96</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>65563,16</t>
+          <t>65670,88</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1792,00</t>
+          <t>1792,45</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>16,27</t>
+          <t>16,44</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -724,7 +724,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-0,62%</t>
+          <t>1,30%</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -737,7 +737,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>88,59</t>
+          <t>91,48</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -750,41 +750,28 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>7520,43</t>
+          <t>7511,35</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Neg Corr</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Divergent</t>
-        </is>
-      </c>
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Fear Greed Index</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Fear Greed Index</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>